<commit_message>
Fix trading module to keep trading balance, last yearly expression
</commit_message>
<xml_diff>
--- a/econ_module/data/h2bb/region_tables.xlsx
+++ b/econ_module/data/h2bb/region_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oliver\Documents\RUB\01_Projekte\IGC_NRW\Arbeitspakete\IGC_model\econ_module\data\h2bb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B93CD7B-7A6F-4454-BF77-68867C344EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4777CE1D-D930-4231-8A9F-A7B67DD88590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-4725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="prices" sheetId="1" r:id="rId1"/>
@@ -163,13 +163,13 @@
     <t>EU-FRA</t>
   </si>
   <si>
-    <t>EU-NDL</t>
-  </si>
-  <si>
     <t>EU-DNK</t>
   </si>
   <si>
     <t>commodity</t>
+  </si>
+  <si>
+    <t>EU-NLD</t>
   </si>
 </sst>
 </file>
@@ -518,7 +518,7 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -856,7 +856,7 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
@@ -946,7 +946,7 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -1054,7 +1054,7 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1392,7 +1392,7 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -1584,9 +1584,7 @@
   <dimension ref="A1:W12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="11" width="4.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="23" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="23" width="4.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.35">
@@ -1594,7 +1592,7 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1932,7 +1930,7 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
@@ -2022,7 +2020,7 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
Introduce supply curve optimization for the trading model v1
</commit_message>
<xml_diff>
--- a/econ_module/data/h2bb/region_tables.xlsx
+++ b/econ_module/data/h2bb/region_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oliver\Documents\RUB\01_Projekte\IGC_NRW\Arbeitspakete\IGC_model\econ_module\data\h2bb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA06AE03-254C-49CD-997E-028E025D78FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E52E6B-DCB5-4294-8890-D2E4E8388DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-4725" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="prices" sheetId="1" r:id="rId1"/>
@@ -353,9 +353,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -725,7 +726,7 @@
         <v>112</v>
       </c>
       <c r="F2" s="1">
-        <f t="shared" ref="F2:S2" si="0">E2+F$8</f>
+        <f t="shared" ref="F2:L2" si="0">E2+F$8</f>
         <v>115</v>
       </c>
       <c r="G2" s="1">
@@ -792,67 +793,67 @@
         <v>1</v>
       </c>
       <c r="D3" s="1">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E3" s="1">
         <f t="shared" ref="E3:L3" si="2">D3+E$8</f>
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F3" s="1">
         <f t="shared" si="2"/>
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G3" s="1">
         <f t="shared" si="2"/>
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H3" s="1">
         <f t="shared" si="2"/>
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I3" s="1">
         <f t="shared" si="2"/>
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="J3" s="1">
         <f t="shared" si="2"/>
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K3" s="1">
         <f t="shared" si="2"/>
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="L3" s="1">
         <f t="shared" si="2"/>
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="M3" s="1">
         <f t="shared" ref="M3:M6" si="3">D3+M$8</f>
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="N3" s="1">
         <f t="shared" ref="N3:S3" si="4">M3+N$8</f>
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="O3" s="1">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="P3" s="1">
         <f t="shared" si="4"/>
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Q3" s="1">
         <f t="shared" si="4"/>
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="R3" s="1">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="S3" s="1">
         <f t="shared" si="4"/>
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.35">
@@ -866,67 +867,67 @@
         <v>1</v>
       </c>
       <c r="D4" s="1">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" ref="E4:L4" si="5">D4+E$8</f>
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="F4" s="1">
         <f t="shared" si="5"/>
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G4" s="1">
         <f t="shared" si="5"/>
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="H4" s="1">
         <f t="shared" si="5"/>
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" si="5"/>
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="J4" s="1">
         <f t="shared" si="5"/>
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K4" s="1">
         <f t="shared" si="5"/>
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="L4" s="1">
         <f t="shared" si="5"/>
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="M4" s="1">
         <f t="shared" si="3"/>
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="N4" s="1">
         <f t="shared" ref="N4:S4" si="6">M4+N$8</f>
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="O4" s="1">
         <f t="shared" si="6"/>
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="P4" s="1">
         <f t="shared" si="6"/>
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="Q4" s="1">
         <f t="shared" si="6"/>
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="R4" s="1">
         <f t="shared" si="6"/>
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="S4" s="1">
         <f t="shared" si="6"/>
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.35">
@@ -1215,67 +1216,67 @@
         <v>1</v>
       </c>
       <c r="D2" s="1">
-        <v>90</v>
+        <v>130</v>
       </c>
       <c r="E2" s="1">
         <f>D2*1.1</f>
-        <v>99.000000000000014</v>
+        <v>143</v>
       </c>
       <c r="F2" s="1">
         <f>D2*1.2</f>
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="G2" s="1">
         <f>D2*1.3</f>
-        <v>117</v>
+        <v>169</v>
       </c>
       <c r="H2" s="1">
         <f>D2*1.4</f>
-        <v>125.99999999999999</v>
+        <v>182</v>
       </c>
       <c r="I2" s="1">
         <f>D2*1.5</f>
-        <v>135</v>
+        <v>195</v>
       </c>
       <c r="J2" s="1">
         <f>D2*1.6</f>
-        <v>144</v>
+        <v>208</v>
       </c>
       <c r="K2" s="1">
         <f>D2*1.8</f>
-        <v>162</v>
+        <v>234</v>
       </c>
       <c r="L2" s="1">
         <f>D2*2</f>
-        <v>180</v>
+        <v>260</v>
       </c>
       <c r="M2" s="1">
         <f>D2*0.9</f>
-        <v>81</v>
+        <v>117</v>
       </c>
       <c r="N2" s="1">
         <f>D2*0.8</f>
-        <v>72</v>
+        <v>104</v>
       </c>
       <c r="O2" s="1">
         <f>D2*0.7</f>
-        <v>62.999999999999993</v>
+        <v>91</v>
       </c>
       <c r="P2" s="1">
         <f>D2*0.6</f>
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="Q2" s="1">
         <f>D2*0.5</f>
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="R2" s="1">
         <f>D2*0.4</f>
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="S2" s="1">
         <f>D2*0.2</f>
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.35">
@@ -1437,67 +1438,67 @@
         <v>1</v>
       </c>
       <c r="D5" s="1">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F5" s="1">
         <f t="shared" si="1"/>
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G5" s="1">
         <f t="shared" si="2"/>
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" si="3"/>
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" si="4"/>
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="J5" s="1">
         <f t="shared" si="5"/>
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="K5" s="1">
         <f t="shared" si="6"/>
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="L5" s="1">
         <f t="shared" si="7"/>
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="M5" s="1">
         <f t="shared" si="8"/>
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="N5" s="1">
         <f t="shared" si="9"/>
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="O5" s="1">
         <f t="shared" si="10"/>
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="P5" s="1">
         <f t="shared" si="11"/>
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="Q5" s="1">
         <f t="shared" si="12"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R5" s="1">
         <f t="shared" si="13"/>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="S5" s="1">
         <f t="shared" si="14"/>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.35">
@@ -1666,66 +1667,66 @@
       <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="2">
         <v>90</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <f>D2*1.1</f>
         <v>99.000000000000014</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="2">
         <f>D2*1.2</f>
         <v>108</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <f>D2*1.3</f>
         <v>117</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <f>D2*1.4</f>
         <v>125.99999999999999</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <f>D2*1.5</f>
         <v>135</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <f>D2*1.6</f>
         <v>144</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <f>D2*1.8</f>
         <v>162</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2" s="2">
         <f>D2*2</f>
         <v>180</v>
       </c>
-      <c r="M2" s="1">
+      <c r="M2" s="2">
         <f>D2*0.9</f>
         <v>81</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <f>D2*0.8</f>
         <v>72</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <f>D2*0.7</f>
         <v>62.999999999999993</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <f>D2*0.6</f>
         <v>54</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <f>D2*0.5</f>
         <v>45</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="2">
         <f>D2*0.4</f>
         <v>36</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="2">
         <f>D2*0.2</f>
         <v>18</v>
       </c>
@@ -1740,66 +1741,66 @@
       <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>10</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <f t="shared" ref="E3:E6" si="0">D3*1.1</f>
         <v>11</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <f t="shared" ref="F3:F6" si="1">D3*1.2</f>
         <v>12</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <f t="shared" ref="G3:G6" si="2">D3*1.3</f>
         <v>13</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <f t="shared" ref="H3:H6" si="3">D3*1.4</f>
         <v>14</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <f t="shared" ref="I3:I6" si="4">D3*1.5</f>
         <v>15</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <f t="shared" ref="J3:J6" si="5">D3*1.6</f>
         <v>16</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <f t="shared" ref="K3:K6" si="6">D3*1.8</f>
         <v>18</v>
       </c>
-      <c r="L3" s="1">
+      <c r="L3" s="2">
         <f t="shared" ref="L3:L6" si="7">D3*2</f>
         <v>20</v>
       </c>
-      <c r="M3" s="1">
+      <c r="M3" s="2">
         <f t="shared" ref="M3:M6" si="8">D3*0.9</f>
         <v>9</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <f t="shared" ref="N3:N6" si="9">D3*0.8</f>
         <v>8</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <f t="shared" ref="O3:O6" si="10">D3*0.7</f>
         <v>7</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <f t="shared" ref="P3:P6" si="11">D3*0.6</f>
         <v>6</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <f t="shared" ref="Q3:Q6" si="12">D3*0.5</f>
         <v>5</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="2">
         <f t="shared" ref="R3:R6" si="13">D3*0.4</f>
         <v>4</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="2">
         <f t="shared" ref="S3:S6" si="14">D3*0.2</f>
         <v>2</v>
       </c>
@@ -1814,68 +1815,68 @@
       <c r="C4" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="1">
-        <v>50</v>
-      </c>
-      <c r="E4" s="1">
+      <c r="D4" s="2">
+        <v>80</v>
+      </c>
+      <c r="E4" s="2">
         <f t="shared" si="0"/>
-        <v>55.000000000000007</v>
-      </c>
-      <c r="F4" s="1">
+        <v>88</v>
+      </c>
+      <c r="F4" s="2">
         <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="G4" s="1">
+        <v>96</v>
+      </c>
+      <c r="G4" s="2">
         <f t="shared" si="2"/>
-        <v>65</v>
-      </c>
-      <c r="H4" s="1">
+        <v>104</v>
+      </c>
+      <c r="H4" s="2">
         <f t="shared" si="3"/>
-        <v>70</v>
-      </c>
-      <c r="I4" s="1">
+        <v>112</v>
+      </c>
+      <c r="I4" s="2">
         <f t="shared" si="4"/>
-        <v>75</v>
-      </c>
-      <c r="J4" s="1">
+        <v>120</v>
+      </c>
+      <c r="J4" s="2">
         <f t="shared" si="5"/>
-        <v>80</v>
-      </c>
-      <c r="K4" s="1">
+        <v>128</v>
+      </c>
+      <c r="K4" s="2">
         <f t="shared" si="6"/>
-        <v>90</v>
-      </c>
-      <c r="L4" s="1">
+        <v>144</v>
+      </c>
+      <c r="L4" s="2">
         <f t="shared" si="7"/>
-        <v>100</v>
-      </c>
-      <c r="M4" s="1">
+        <v>160</v>
+      </c>
+      <c r="M4" s="2">
         <f t="shared" si="8"/>
-        <v>45</v>
-      </c>
-      <c r="N4" s="1">
+        <v>72</v>
+      </c>
+      <c r="N4" s="2">
         <f t="shared" si="9"/>
+        <v>64</v>
+      </c>
+      <c r="O4" s="2">
+        <f t="shared" si="10"/>
+        <v>56</v>
+      </c>
+      <c r="P4" s="2">
+        <f t="shared" si="11"/>
+        <v>48</v>
+      </c>
+      <c r="Q4" s="2">
+        <f t="shared" si="12"/>
         <v>40</v>
       </c>
-      <c r="O4" s="1">
-        <f t="shared" si="10"/>
-        <v>35</v>
-      </c>
-      <c r="P4" s="1">
-        <f t="shared" si="11"/>
-        <v>30</v>
-      </c>
-      <c r="Q4" s="1">
-        <f t="shared" si="12"/>
-        <v>25</v>
-      </c>
-      <c r="R4" s="1">
+      <c r="R4" s="2">
         <f t="shared" si="13"/>
-        <v>20</v>
-      </c>
-      <c r="S4" s="1">
+        <v>32</v>
+      </c>
+      <c r="S4" s="2">
         <f t="shared" si="14"/>
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.35">
@@ -1888,66 +1889,66 @@
       <c r="C5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>30</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="2">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <f t="shared" si="2"/>
         <v>39</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <f t="shared" si="3"/>
         <v>42</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <f t="shared" si="4"/>
         <v>45</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <f t="shared" si="5"/>
         <v>48</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <f t="shared" si="6"/>
         <v>54</v>
       </c>
-      <c r="L5" s="1">
+      <c r="L5" s="2">
         <f t="shared" si="7"/>
         <v>60</v>
       </c>
-      <c r="M5" s="1">
+      <c r="M5" s="2">
         <f t="shared" si="8"/>
         <v>27</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <f t="shared" si="9"/>
         <v>24</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <f t="shared" si="10"/>
         <v>21</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <f t="shared" si="11"/>
         <v>18</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <f t="shared" si="12"/>
         <v>15</v>
       </c>
-      <c r="R5" s="1">
+      <c r="R5" s="2">
         <f t="shared" si="13"/>
         <v>12</v>
       </c>
-      <c r="S5" s="1">
+      <c r="S5" s="2">
         <f t="shared" si="14"/>
         <v>6</v>
       </c>
@@ -1962,66 +1963,66 @@
       <c r="C6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
         <v>20</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="2">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <f t="shared" si="2"/>
         <v>26</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <f t="shared" si="3"/>
         <v>28</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <f t="shared" si="4"/>
         <v>30</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <f t="shared" si="5"/>
         <v>32</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <f t="shared" si="6"/>
         <v>36</v>
       </c>
-      <c r="L6" s="1">
+      <c r="L6" s="2">
         <f t="shared" si="7"/>
         <v>40</v>
       </c>
-      <c r="M6" s="1">
+      <c r="M6" s="2">
         <f t="shared" si="8"/>
         <v>18</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <f t="shared" si="9"/>
         <v>16</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <f t="shared" si="10"/>
         <v>14</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <f t="shared" si="11"/>
         <v>12</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <f t="shared" si="12"/>
         <v>10</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="2">
         <f t="shared" si="13"/>
         <v>8</v>
       </c>
-      <c r="S6" s="1">
+      <c r="S6" s="2">
         <f t="shared" si="14"/>
         <v>4</v>
       </c>

</xml_diff>